<commit_message>
feat: align BBCH stage runtime rules and publish missing frontend API docs
</commit_message>
<xml_diff>
--- a/docs/生育期code_list.xlsx
+++ b/docs/生育期code_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\workspace\CropFlow\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B93EF9C-D3C7-4327-A2A6-878BBECC02E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7F886D8-D50B-4870-BF6A-989AF51E94AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{901ADA71-5632-4438-A5AE-820A0E0A3559}"/>
+    <workbookView xWindow="13920" yWindow="1485" windowWidth="10635" windowHeight="14235" xr2:uid="{901ADA71-5632-4438-A5AE-820A0E0A3559}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="131">
   <si>
     <t>成长阶段</t>
   </si>
@@ -1460,15 +1460,9 @@
     <t>再生季孕穗期</t>
   </si>
   <si>
-    <t>Z21</t>
-  </si>
-  <si>
     <t>孕穗早期：再生苗幼穗分化达到5期，剑叶叶枕还在倒二叶叶鞘内，距倒二叶叶枕5cm以内</t>
   </si>
   <si>
-    <t>Z23</t>
-  </si>
-  <si>
     <r>
       <t>再生苗幼穗分化达到</t>
     </r>
@@ -1512,106 +1506,134 @@
     </r>
   </si>
   <si>
-    <t>Z25</t>
-  </si>
-  <si>
     <t>孕穗中期：再生苗幼穗分化达到7期，剑叶叶枕伸出倒二叶5~10cm</t>
   </si>
   <si>
-    <t>Z27</t>
-  </si>
-  <si>
     <t>孕穗后期：再生苗幼穗分化达到8期，剑叶叶枕伸出倒二叶叶枕10cm以上</t>
   </si>
   <si>
     <t>再生季抽穗期</t>
   </si>
   <si>
-    <t>Z30</t>
-  </si>
-  <si>
     <t>再生季破口</t>
   </si>
   <si>
-    <t>Z31</t>
-  </si>
-  <si>
     <t>再生季10%的穗抽出</t>
   </si>
   <si>
-    <t>Z32</t>
-  </si>
-  <si>
     <t>再生季20%的穗抽出</t>
   </si>
   <si>
-    <t>Z33</t>
-  </si>
-  <si>
     <t>再生季30%的穗抽出</t>
   </si>
   <si>
-    <t>Z34</t>
-  </si>
-  <si>
     <t>再生季40%的穗抽出</t>
   </si>
   <si>
-    <t>Z35</t>
-  </si>
-  <si>
     <t>再生季50%的穗抽出</t>
   </si>
   <si>
-    <t>Z36</t>
-  </si>
-  <si>
     <t>再生季60%的穗抽出</t>
   </si>
   <si>
-    <t>Z37</t>
-  </si>
-  <si>
     <t>再生季70%的穗抽出</t>
   </si>
   <si>
-    <t>Z38</t>
-  </si>
-  <si>
     <t>再生季80%的穗抽出</t>
   </si>
   <si>
-    <t>Z39</t>
-  </si>
-  <si>
     <t>再生穗完全抽出</t>
   </si>
   <si>
     <t>再生季灌浆成熟期</t>
   </si>
   <si>
-    <t>Z41</t>
-  </si>
-  <si>
     <t>乳熟：稻穗开始灌浆，稻穗呈绿色，50%以上稻穗籽粒未充实变硬</t>
   </si>
   <si>
-    <t>Z43</t>
-  </si>
-  <si>
     <t>蜡熟：稻穗50%以上籽粒变硬，稻穗由绿逐渐变黄，黄熟度在50%以下</t>
   </si>
   <si>
+    <t>黄熟：稻穗90%以上籽粒变硬，黄熟度在90%</t>
+  </si>
+  <si>
+    <t>完熟：稻穗95%以上籽粒变硬，黄熟度在95%以上。</t>
+  </si>
+  <si>
+    <t>孕穗</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
     <t>Z45</t>
-  </si>
-  <si>
-    <t>黄熟：稻穗90%以上籽粒变硬，黄熟度在90%</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z46</t>
+    <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
     <t>Z47</t>
-  </si>
-  <si>
-    <t>完熟：稻穗95%以上籽粒变硬，黄熟度在95%以上。</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z48</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z50</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z51</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z52</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z53</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z54</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z55</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z56</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z57</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z58</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z59</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z81</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z83</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z89</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Z90</t>
+    <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1796,15 +1818,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1821,6 +1834,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2137,7 +2159,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B21CAED-4E62-4EE6-831D-D5F97412B1C7}">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="30.375" customWidth="1"/>
@@ -2155,7 +2177,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3">
@@ -2166,7 +2188,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13"/>
+      <c r="A3" s="10"/>
       <c r="B3" s="3">
         <v>1</v>
       </c>
@@ -2175,7 +2197,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13"/>
+      <c r="A4" s="10"/>
       <c r="B4" s="3">
         <v>3</v>
       </c>
@@ -2184,7 +2206,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13"/>
+      <c r="A5" s="10"/>
       <c r="B5" s="3">
         <v>5</v>
       </c>
@@ -2193,7 +2215,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13"/>
+      <c r="A6" s="10"/>
       <c r="B6" s="3">
         <v>6</v>
       </c>
@@ -2202,7 +2224,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="3">
         <v>7</v>
       </c>
@@ -2211,7 +2233,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="3">
         <v>9</v>
       </c>
@@ -2220,7 +2242,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="9" t="s">
         <v>11</v>
       </c>
       <c r="B9" s="3">
@@ -2231,7 +2253,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13"/>
+      <c r="A10" s="10"/>
       <c r="B10" s="3">
         <v>11</v>
       </c>
@@ -2240,7 +2262,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="13"/>
+      <c r="A11" s="10"/>
       <c r="B11" s="3">
         <v>12</v>
       </c>
@@ -2249,7 +2271,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="13"/>
+      <c r="A12" s="10"/>
       <c r="B12" s="3">
         <v>13</v>
       </c>
@@ -2258,7 +2280,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="13"/>
+      <c r="A13" s="10"/>
       <c r="B13" s="3" t="s">
         <v>16</v>
       </c>
@@ -2267,7 +2289,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14"/>
+      <c r="A14" s="11"/>
       <c r="B14" s="3">
         <v>19</v>
       </c>
@@ -2276,7 +2298,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B15" s="3">
@@ -2287,7 +2309,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="13"/>
+      <c r="A16" s="10"/>
       <c r="B16" s="3">
         <v>22</v>
       </c>
@@ -2295,8 +2317,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="13"/>
+    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10"/>
       <c r="B17" s="3">
         <v>23</v>
       </c>
@@ -2304,8 +2326,8 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="13"/>
+    <row r="18" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="10"/>
       <c r="B18" s="3" t="s">
         <v>23</v>
       </c>
@@ -2313,8 +2335,8 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="13"/>
+    <row r="19" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="10"/>
       <c r="B19" s="3">
         <v>29</v>
       </c>
@@ -2322,8 +2344,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="13"/>
+    <row r="20" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="10"/>
       <c r="B20" s="3">
         <v>210</v>
       </c>
@@ -2331,8 +2353,8 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="14"/>
+    <row r="21" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="11"/>
       <c r="B21" s="3">
         <v>211</v>
       </c>
@@ -2340,8 +2362,8 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
+    <row r="22" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
         <v>27</v>
       </c>
       <c r="B22" s="3">
@@ -2351,8 +2373,8 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="30" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="13"/>
+    <row r="23" spans="1:4" ht="30" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="10"/>
       <c r="B23" s="3">
         <v>31</v>
       </c>
@@ -2360,8 +2382,8 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="13"/>
+    <row r="24" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="10"/>
       <c r="B24" s="3">
         <v>32</v>
       </c>
@@ -2369,8 +2391,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="13"/>
+    <row r="25" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
       <c r="B25" s="3" t="s">
         <v>23</v>
       </c>
@@ -2378,8 +2400,8 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="13"/>
+    <row r="26" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="10"/>
       <c r="B26" s="3">
         <v>38</v>
       </c>
@@ -2387,8 +2409,8 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="14"/>
+    <row r="27" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="11"/>
       <c r="B27" s="3">
         <v>39</v>
       </c>
@@ -2396,8 +2418,8 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="74.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="12" t="s">
+    <row r="28" spans="1:4" ht="74.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="9" t="s">
         <v>33</v>
       </c>
       <c r="B28" s="3">
@@ -2407,8 +2429,8 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="60" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="13"/>
+    <row r="29" spans="1:4" ht="60" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="10"/>
       <c r="B29" s="3">
         <v>42</v>
       </c>
@@ -2416,8 +2438,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="13"/>
+    <row r="30" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="10"/>
       <c r="B30" s="3">
         <v>43</v>
       </c>
@@ -2425,8 +2447,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="60.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="13"/>
+    <row r="31" spans="1:4" ht="60.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="10"/>
       <c r="B31" s="3">
         <v>44</v>
       </c>
@@ -2434,17 +2456,20 @@
         <v>37</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="60.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="13"/>
+    <row r="32" spans="1:4" ht="60.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="10"/>
       <c r="B32" s="3">
         <v>45</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>38</v>
       </c>
+      <c r="D32" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="33" spans="1:3" ht="72.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="13"/>
+      <c r="A33" s="10"/>
       <c r="B33" s="3">
         <v>46</v>
       </c>
@@ -2453,7 +2478,7 @@
       </c>
     </row>
     <row r="34" spans="1:3" ht="59.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="13"/>
+      <c r="A34" s="10"/>
       <c r="B34" s="3">
         <v>47</v>
       </c>
@@ -2462,7 +2487,7 @@
       </c>
     </row>
     <row r="35" spans="1:3" ht="87" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="14"/>
+      <c r="A35" s="11"/>
       <c r="B35" s="3">
         <v>48</v>
       </c>
@@ -2471,7 +2496,7 @@
       </c>
     </row>
     <row r="36" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="15" t="s">
+      <c r="A36" s="12" t="s">
         <v>42</v>
       </c>
       <c r="B36" s="6">
@@ -2482,7 +2507,7 @@
       </c>
     </row>
     <row r="37" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="16"/>
+      <c r="A37" s="13"/>
       <c r="B37" s="3">
         <v>52</v>
       </c>
@@ -2491,7 +2516,7 @@
       </c>
     </row>
     <row r="38" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="16"/>
+      <c r="A38" s="13"/>
       <c r="B38" s="3">
         <v>53</v>
       </c>
@@ -2500,7 +2525,7 @@
       </c>
     </row>
     <row r="39" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="16"/>
+      <c r="A39" s="13"/>
       <c r="B39" s="3">
         <v>54</v>
       </c>
@@ -2509,7 +2534,7 @@
       </c>
     </row>
     <row r="40" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="16"/>
+      <c r="A40" s="13"/>
       <c r="B40" s="6">
         <v>55</v>
       </c>
@@ -2518,7 +2543,7 @@
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="16"/>
+      <c r="A41" s="13"/>
       <c r="B41" s="3">
         <v>56</v>
       </c>
@@ -2527,7 +2552,7 @@
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="16"/>
+      <c r="A42" s="13"/>
       <c r="B42" s="3">
         <v>57</v>
       </c>
@@ -2536,7 +2561,7 @@
       </c>
     </row>
     <row r="43" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="16"/>
+      <c r="A43" s="13"/>
       <c r="B43" s="6">
         <v>58</v>
       </c>
@@ -2545,7 +2570,7 @@
       </c>
     </row>
     <row r="44" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="17"/>
+      <c r="A44" s="14"/>
       <c r="B44" s="3">
         <v>59</v>
       </c>
@@ -2554,7 +2579,7 @@
       </c>
     </row>
     <row r="45" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="12" t="s">
+      <c r="A45" s="9" t="s">
         <v>52</v>
       </c>
       <c r="B45" s="3">
@@ -2565,7 +2590,7 @@
       </c>
     </row>
     <row r="46" spans="1:3" ht="30" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="13"/>
+      <c r="A46" s="10"/>
       <c r="B46" s="3">
         <v>63</v>
       </c>
@@ -2574,7 +2599,7 @@
       </c>
     </row>
     <row r="47" spans="1:3" ht="30" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="13"/>
+      <c r="A47" s="10"/>
       <c r="B47" s="3">
         <v>64</v>
       </c>
@@ -2583,7 +2608,7 @@
       </c>
     </row>
     <row r="48" spans="1:3" ht="30" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="13"/>
+      <c r="A48" s="10"/>
       <c r="B48" s="3">
         <v>65</v>
       </c>
@@ -2592,7 +2617,7 @@
       </c>
     </row>
     <row r="49" spans="1:3" ht="44.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="14"/>
+      <c r="A49" s="11"/>
       <c r="B49" s="3">
         <v>69</v>
       </c>
@@ -2601,7 +2626,7 @@
       </c>
     </row>
     <row r="50" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="12" t="s">
+      <c r="A50" s="9" t="s">
         <v>58</v>
       </c>
       <c r="B50" s="3">
@@ -2612,7 +2637,7 @@
       </c>
     </row>
     <row r="51" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="13"/>
+      <c r="A51" s="10"/>
       <c r="B51" s="3">
         <v>73</v>
       </c>
@@ -2621,7 +2646,7 @@
       </c>
     </row>
     <row r="52" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="13"/>
+      <c r="A52" s="10"/>
       <c r="B52" s="3">
         <v>75</v>
       </c>
@@ -2630,7 +2655,7 @@
       </c>
     </row>
     <row r="53" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="14"/>
+      <c r="A53" s="11"/>
       <c r="B53" s="3">
         <v>77</v>
       </c>
@@ -2639,7 +2664,7 @@
       </c>
     </row>
     <row r="54" spans="1:3" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="12" t="s">
+      <c r="A54" s="9" t="s">
         <v>63</v>
       </c>
       <c r="B54" s="3">
@@ -2650,7 +2675,7 @@
       </c>
     </row>
     <row r="55" spans="1:3" ht="86.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="13"/>
+      <c r="A55" s="10"/>
       <c r="B55" s="3">
         <v>85</v>
       </c>
@@ -2659,7 +2684,7 @@
       </c>
     </row>
     <row r="56" spans="1:3" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="13"/>
+      <c r="A56" s="10"/>
       <c r="B56" s="3">
         <v>87</v>
       </c>
@@ -2668,7 +2693,7 @@
       </c>
     </row>
     <row r="57" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="14"/>
+      <c r="A57" s="11"/>
       <c r="B57" s="3">
         <v>89</v>
       </c>
@@ -2677,7 +2702,7 @@
       </c>
     </row>
     <row r="58" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="12" t="s">
+      <c r="A58" s="9" t="s">
         <v>68</v>
       </c>
       <c r="B58" s="3">
@@ -2688,7 +2713,7 @@
       </c>
     </row>
     <row r="59" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="13"/>
+      <c r="A59" s="10"/>
       <c r="B59" s="3">
         <v>97</v>
       </c>
@@ -2697,7 +2722,7 @@
       </c>
     </row>
     <row r="60" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="14"/>
+      <c r="A60" s="11"/>
       <c r="B60" s="3">
         <v>99</v>
       </c>
@@ -2706,7 +2731,7 @@
       </c>
     </row>
     <row r="61" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="9" t="s">
+      <c r="A61" s="15" t="s">
         <v>72</v>
       </c>
       <c r="B61" s="3" t="s">
@@ -2717,7 +2742,7 @@
       </c>
     </row>
     <row r="62" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="11"/>
+      <c r="A62" s="17"/>
       <c r="B62" s="3" t="s">
         <v>75</v>
       </c>
@@ -2726,7 +2751,7 @@
       </c>
     </row>
     <row r="63" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="9" t="s">
+      <c r="A63" s="15" t="s">
         <v>77</v>
       </c>
       <c r="B63" s="3" t="s">
@@ -2737,7 +2762,7 @@
       </c>
     </row>
     <row r="64" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="10"/>
+      <c r="A64" s="16"/>
       <c r="B64" s="3" t="s">
         <v>80</v>
       </c>
@@ -2746,7 +2771,7 @@
       </c>
     </row>
     <row r="65" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="11"/>
+      <c r="A65" s="17"/>
       <c r="B65" s="3" t="s">
         <v>82</v>
       </c>
@@ -2755,7 +2780,7 @@
       </c>
     </row>
     <row r="66" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="9" t="s">
+      <c r="A66" s="15" t="s">
         <v>84</v>
       </c>
       <c r="B66" s="3" t="s">
@@ -2766,7 +2791,7 @@
       </c>
     </row>
     <row r="67" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="10"/>
+      <c r="A67" s="16"/>
       <c r="B67" s="3" t="s">
         <v>87</v>
       </c>
@@ -2775,7 +2800,7 @@
       </c>
     </row>
     <row r="68" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="11"/>
+      <c r="A68" s="17"/>
       <c r="B68" s="3" t="s">
         <v>89</v>
       </c>
@@ -2784,175 +2809,183 @@
       </c>
     </row>
     <row r="69" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="9" t="s">
+      <c r="A69" s="15" t="s">
         <v>91</v>
       </c>
       <c r="B69" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C69" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C69" s="4" t="s">
+    </row>
+    <row r="70" spans="1:3" ht="45" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="16"/>
+      <c r="B70" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C70" s="4" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="45" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="10"/>
-      <c r="B70" s="3" t="s">
+    <row r="71" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="16"/>
+      <c r="B71" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C71" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C70" s="4" t="s">
+    </row>
+    <row r="72" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="17"/>
+      <c r="B72" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C72" s="4" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="10"/>
-      <c r="B71" s="3" t="s">
+    <row r="73" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="C71" s="4" t="s">
+      <c r="B73" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C73" s="4" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="11"/>
-      <c r="B72" s="3" t="s">
+    <row r="74" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="16"/>
+      <c r="B74" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C74" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C72" s="4" t="s">
+    </row>
+    <row r="75" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="16"/>
+      <c r="B75" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C75" s="4" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="9" t="s">
+    <row r="76" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="16"/>
+      <c r="B76" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C76" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B73" s="3" t="s">
+    </row>
+    <row r="77" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="16"/>
+      <c r="B77" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C77" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C73" s="4" t="s">
+    </row>
+    <row r="78" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="16"/>
+      <c r="B78" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C78" s="4" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="10"/>
-      <c r="B74" s="3" t="s">
+    <row r="79" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="16"/>
+      <c r="B79" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C79" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C74" s="4" t="s">
+    </row>
+    <row r="80" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="16"/>
+      <c r="B80" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C80" s="4" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="10"/>
-      <c r="B75" s="3" t="s">
+    <row r="81" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="16"/>
+      <c r="B81" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C81" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C75" s="4" t="s">
+    </row>
+    <row r="82" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="17"/>
+      <c r="B82" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C82" s="4" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="10"/>
-      <c r="B76" s="3" t="s">
+    <row r="83" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="C76" s="4" t="s">
+      <c r="B83" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C83" s="4" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="10"/>
-      <c r="B77" s="3" t="s">
+    <row r="84" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="16"/>
+      <c r="B84" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C84" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="C77" s="4" t="s">
+    </row>
+    <row r="85" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="16"/>
+      <c r="B85" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C85" s="4" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="10"/>
-      <c r="B78" s="3" t="s">
+    <row r="86" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="17"/>
+      <c r="B86" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C86" s="4" t="s">
         <v>111</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="10"/>
-      <c r="B79" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="10"/>
-      <c r="B80" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C80" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="10"/>
-      <c r="B81" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C81" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="11"/>
-      <c r="B82" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C82" s="4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="C83" s="4" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="10"/>
-      <c r="B84" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C84" s="4" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="10"/>
-      <c r="B85" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="C85" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="11"/>
-      <c r="B86" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C86" s="4" t="s">
-        <v>129</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A73:A82"/>
+    <mergeCell ref="A83:A86"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A58:A60"/>
+    <mergeCell ref="A61:A62"/>
+    <mergeCell ref="A63:A65"/>
+    <mergeCell ref="A66:A68"/>
+    <mergeCell ref="A69:A72"/>
     <mergeCell ref="A45:A49"/>
     <mergeCell ref="A28:A35"/>
     <mergeCell ref="A54:A57"/>
@@ -2961,14 +2994,6 @@
     <mergeCell ref="A15:A21"/>
     <mergeCell ref="A22:A27"/>
     <mergeCell ref="A36:A44"/>
-    <mergeCell ref="A73:A82"/>
-    <mergeCell ref="A83:A86"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A58:A60"/>
-    <mergeCell ref="A61:A62"/>
-    <mergeCell ref="A63:A65"/>
-    <mergeCell ref="A66:A68"/>
-    <mergeCell ref="A69:A72"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>